<commit_message>
feat: implement utility bill OCR and carbon analysis
</commit_message>
<xml_diff>
--- a/data/category_carbon.xlsx
+++ b/data/category_carbon.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mcbri\PycharmProjects\GreenStep\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\home\Desktop\ai-server\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC5C347E-5677-4861-A082-E34DC893033C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47B85ACB-5BD9-4EEF-86C6-6B217A521203}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0F6C9620-84A5-47F2-85DD-B3E6F7730BB0}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{0F6C9620-84A5-47F2-85DD-B3E6F7730BB0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="90">
   <si>
     <t xml:space="preserve">메인 카테고리 </t>
   </si>
@@ -299,6 +300,11 @@
   </si>
   <si>
     <t>전기차충전</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">가정에너지
+</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -351,7 +357,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -360,6 +366,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -379,9 +388,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 테마">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -419,7 +428,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -525,7 +534,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -667,7 +676,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -676,15 +685,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D01474DA-6137-4A88-9E69-40BEBEAA13F3}">
   <dimension ref="A1:D76"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="21.19921875" customWidth="1"/>
-    <col min="2" max="2" width="16.796875" customWidth="1"/>
-    <col min="3" max="3" width="25.09765625" customWidth="1"/>
-    <col min="4" max="4" width="32.796875" customWidth="1"/>
+    <col min="1" max="1" width="21.1640625" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="25.08203125" customWidth="1"/>
+    <col min="4" max="4" width="32.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -698,7 +707,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -709,7 +718,7 @@
         <v>2.647422E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -720,7 +729,7 @@
         <v>1.9284400000000001E-4</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -731,9 +740,9 @@
         <v>2.5380369999999999E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A5" t="s">
-        <v>4</v>
+    <row r="5" spans="1:4" ht="34" x14ac:dyDescent="0.45">
+      <c r="A5" s="3" t="s">
+        <v>89</v>
       </c>
       <c r="B5" t="s">
         <v>8</v>
@@ -745,7 +754,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -756,7 +765,7 @@
         <v>1.6655000000000001E-4</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -767,7 +776,7 @@
         <v>1.3629000000000001E-4</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -778,7 +787,7 @@
         <v>2.6499999999999999E-4</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -789,7 +798,7 @@
         <v>2.849E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -800,7 +809,7 @@
         <v>1.316843E-3</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -811,7 +820,7 @@
         <v>1.1250030000000001E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -822,7 +831,7 @@
         <v>1.1525999999999999E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>82</v>
       </c>
@@ -833,7 +842,7 @@
         <v>1.5523100000000001E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>82</v>
       </c>
@@ -844,7 +853,7 @@
         <v>1.2313100000000001E-4</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>15</v>
       </c>
@@ -855,7 +864,7 @@
         <v>5.1858299999999998E-5</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -866,7 +875,7 @@
         <v>2.9560700000000001E-7</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -877,7 +886,7 @@
         <v>1.43545E-4</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>19</v>
       </c>
@@ -888,7 +897,7 @@
         <v>1.3899999999999999E-4</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>19</v>
       </c>
@@ -899,7 +908,7 @@
         <v>4.6548999999999999E-4</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -910,7 +919,7 @@
         <v>1.8830999999999999E-4</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>19</v>
       </c>
@@ -921,7 +930,7 @@
         <v>2.42477E-4</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>19</v>
       </c>
@@ -932,7 +941,7 @@
         <v>2.3713E-4</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>25</v>
       </c>
@@ -943,7 +952,7 @@
         <v>1.5415000000000001E-4</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>25</v>
       </c>
@@ -954,7 +963,7 @@
         <v>2.1644490000000001E-3</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>25</v>
       </c>
@@ -965,7 +974,7 @@
         <v>1.8150999999999999E-4</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>25</v>
       </c>
@@ -976,7 +985,7 @@
         <v>3.6999999999999998E-5</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>25</v>
       </c>
@@ -987,7 +996,7 @@
         <v>1.6750000000000001E-4</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>25</v>
       </c>
@@ -998,7 +1007,7 @@
         <v>4.7367999999999998E-4</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>25</v>
       </c>
@@ -1009,7 +1018,7 @@
         <v>6.6000000000000005E-5</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>25</v>
       </c>
@@ -1020,7 +1029,7 @@
         <v>8.9099999999999997E-5</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>34</v>
       </c>
@@ -1031,7 +1040,7 @@
         <v>2.6403E-4</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>34</v>
       </c>
@@ -1042,7 +1051,7 @@
         <v>4.057E-4</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>34</v>
       </c>
@@ -1053,7 +1062,7 @@
         <v>1.1325E-4</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
         <v>34</v>
       </c>
@@ -1064,7 +1073,7 @@
         <v>3.0180000000000002E-4</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
         <v>34</v>
       </c>
@@ -1075,7 +1084,7 @@
         <v>4.2185999999999998E-4</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
         <v>34</v>
       </c>
@@ -1086,7 +1095,7 @@
         <v>1.5634000000000001E-4</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
         <v>34</v>
       </c>
@@ -1097,7 +1106,7 @@
         <v>1.0906E-4</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
         <v>34</v>
       </c>
@@ -1108,7 +1117,7 @@
         <v>1.7741E-4</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
         <v>34</v>
       </c>
@@ -1119,7 +1128,7 @@
         <v>7.6719999999999997E-5</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
         <v>34</v>
       </c>
@@ -1130,7 +1139,7 @@
         <v>1.4584E-4</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
         <v>34</v>
       </c>
@@ -1141,7 +1150,7 @@
         <v>2.1641999999999999E-4</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
         <v>34</v>
       </c>
@@ -1152,7 +1161,7 @@
         <v>2.8778000000000001E-4</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
         <v>34</v>
       </c>
@@ -1163,7 +1172,7 @@
         <v>2.1458999999999999E-4</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
         <v>34</v>
       </c>
@@ -1174,7 +1183,7 @@
         <v>2.9749000000000003E-4</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
         <v>34</v>
       </c>
@@ -1185,7 +1194,7 @@
         <v>2.3188000000000001E-4</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
         <v>34</v>
       </c>
@@ -1196,7 +1205,7 @@
         <v>7.1740000000000001E-5</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
         <v>34</v>
       </c>
@@ -1207,7 +1216,7 @@
         <v>9.8880000000000002E-5</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
         <v>34</v>
       </c>
@@ -1218,7 +1227,7 @@
         <v>1.3993999999999999E-4</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
         <v>34</v>
       </c>
@@ -1229,7 +1238,7 @@
         <v>1.6992999999999999E-4</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
         <v>34</v>
       </c>
@@ -1240,7 +1249,7 @@
         <v>1.9523000000000001E-4</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
         <v>34</v>
       </c>
@@ -1251,7 +1260,7 @@
         <v>3.4260000000000001E-5</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
         <v>34</v>
       </c>
@@ -1262,7 +1271,7 @@
         <v>9.4469999999999995E-5</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
         <v>34</v>
       </c>
@@ -1273,7 +1282,7 @@
         <v>7.9870000000000006E-5</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
         <v>34</v>
       </c>
@@ -1284,7 +1293,7 @@
         <v>4.2034E-4</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
         <v>34</v>
       </c>
@@ -1295,7 +1304,7 @@
         <v>1.4292999999999999E-4</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
         <v>34</v>
       </c>
@@ -1306,7 +1315,7 @@
         <v>1.8310000000000001E-4</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
         <v>34</v>
       </c>
@@ -1317,7 +1326,7 @@
         <v>1.2370999999999999E-4</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
         <v>34</v>
       </c>
@@ -1328,7 +1337,7 @@
         <v>1.4839000000000001E-4</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
         <v>34</v>
       </c>
@@ -1339,7 +1348,7 @@
         <v>1.6006000000000001E-4</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
         <v>34</v>
       </c>
@@ -1350,7 +1359,7 @@
         <v>4.2599999999999999E-5</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
         <v>34</v>
       </c>
@@ -1361,7 +1370,7 @@
         <v>2.7608E-4</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A62" t="s">
         <v>34</v>
       </c>
@@ -1372,7 +1381,7 @@
         <v>3.4262000000000002E-4</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
         <v>34</v>
       </c>
@@ -1383,7 +1392,7 @@
         <v>1.0378999999999999E-4</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A64" t="s">
         <v>34</v>
       </c>
@@ -1394,7 +1403,7 @@
         <v>8.6840000000000002E-5</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A65" t="s">
         <v>34</v>
       </c>
@@ -1405,7 +1414,7 @@
         <v>4.7663000000000002E-4</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A66" t="s">
         <v>34</v>
       </c>
@@ -1416,7 +1425,7 @@
         <v>8.9679999999999995E-5</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A67" t="s">
         <v>34</v>
       </c>
@@ -1427,7 +1436,7 @@
         <v>1.2488000000000001E-4</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A68" t="s">
         <v>34</v>
       </c>
@@ -1438,7 +1447,7 @@
         <v>1.0665E-4</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A69" t="s">
         <v>34</v>
       </c>
@@ -1449,7 +1458,7 @@
         <v>1.5142000000000001E-4</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A70" t="s">
         <v>34</v>
       </c>
@@ -1460,7 +1469,7 @@
         <v>1.9165E-4</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A71" t="s">
         <v>34</v>
       </c>
@@ -1471,7 +1480,7 @@
         <v>5.6390000000000001E-5</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A72" t="s">
         <v>34</v>
       </c>
@@ -1482,7 +1491,7 @@
         <v>1.1496E-4</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A73" t="s">
         <v>34</v>
       </c>
@@ -1493,7 +1502,7 @@
         <v>8.4740000000000005E-5</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A74" t="s">
         <v>34</v>
       </c>
@@ -1504,7 +1513,7 @@
         <v>6.4460000000000003E-5</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A75" t="s">
         <v>34</v>
       </c>
@@ -1515,7 +1524,7 @@
         <v>8.6609999999999999E-5</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A76" t="s">
         <v>79</v>
       </c>
@@ -1531,4 +1540,14 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEE9014C-D6DC-4E20-96D9-F9335A2245D6}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <sheetData/>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>